<commit_message>
Quita el reto de Juice Shop sin evidencia (punto 7 del segundo corte)
No hay captura del reto, así que se retiran la mención en clase/notas.md, la fila T7
de la tabla de clase y la referencia a OWASP Juice Shop, que ya no se cita.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wXTRos7KirxghfoUX112D
</commit_message>
<xml_diff>
--- a/clase/tabla-stride-clase.xlsx
+++ b/clase/tabla-stride-clase.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -907,68 +907,6 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Formulario de login (reto práctico OWASP Juice Shop)</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Spoofing</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Se logró iniciar sesión como administrador sin conocer su contraseña, explotando la ausencia de consultas parametrizadas en el formulario de login.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Se ejecutó el reto guiado #1 de la sección 4 de la guía del taller (inyección en el campo de login) contra la instancia local de Juice Shop en Docker.</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Alto — control total de la cuenta de administrador</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Alta (confirmado en laboratorio)</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Sin prepared statements ni validación de input en el campo de login (confirmado en laboratorio).</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Usar consultas parametrizadas / ORM; nunca concatenar el input del usuario directamente en una consulta SQL</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Equipo de Seguridad</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Confirmado en laboratorio</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>